<commit_message>
refactor(xlsx): fix inefficiencies and improve tests
Fix inefficiencies, bugs, and improve code quality in comment extraction.
Support modern comments, in addition to notes, with direct XML parsing.
Add security hardening to prevent XXE attacks.
Extend and improve tests.
Regenerate groundtruth files.

Signed-off-by: Cesar Berrospi Ramis <ceb@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/tests/data/xlsx/xlsx_comments.xlsx
+++ b/tests/data/xlsx/xlsx_comments.xlsx
@@ -1,34 +1,153 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ceb/git/docling-3/tests/data/xlsx/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED46F2A-5D23-D74E-B2A0-4FAF268BC642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="10860" yWindow="2920" windowWidth="34560" windowHeight="22340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>John Reviewer</author>
+    <author>Jane Editor</author>
+    <author>tc={04C1C54B-2744-A647-93D1-A99C27C7EFDC}</author>
+    <author>tc={3A26E9AE-8B38-864D-BAF4-BA5D9C6E1DA4}</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Why Python specifically?</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B2" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Which libraries are you referring to?</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F7" authorId="2" shapeId="0" xr:uid="{04C1C54B-2744-A647-93D1-A99C27C7EFDC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Minimum number of saltwater ducks
+Reply:
+    I never thought it would be so low</t>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="3" shapeId="0" xr:uid="{3A26E9AE-8B38-864D-BAF4-BA5D9C6E1DA4}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Maximum number of ducks</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Python is great</t>
+  </si>
+  <si>
+    <t>Machine learning libraries</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Freshwater Ducks</t>
+  </si>
+  <si>
+    <t>Saltwater Ducks</t>
+  </si>
+  <si>
+    <t>Ducks</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,103 +165,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>John Reviewer</author>
-    <author>Jane Editor</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Why Python specifically?</t>
-      </text>
-    </comment>
-    <comment ref="B2" authorId="1" shapeId="0">
-      <text>
-        <t>Which libraries are you referring to?</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Jane Smith (JS)" id="{ED88F4F5-A552-4A41-970D-6B23DC2319F4}" userId="Jane Smith (JS)" providerId="None"/>
+  <person displayName="Marcus Sterling (MS)" id="{F91C2EA4-71EE-4B4A-B219-115641A7AB48}" userId="Marcus Sterling (MS)" providerId="None"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -428,31 +476,135 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="F7" dT="2026-06-18T17:12:37.41" personId="{ED88F4F5-A552-4A41-970D-6B23DC2319F4}" id="{04C1C54B-2744-A647-93D1-A99C27C7EFDC}">
+    <text>Minimum number of saltwater ducks</text>
+  </threadedComment>
+  <threadedComment ref="F7" dT="2026-06-18T17:15:52.31" personId="{F91C2EA4-71EE-4B4A-B219-115641A7AB48}" id="{9079903E-5C85-DC40-828F-9D93A620480C}" parentId="{04C1C54B-2744-A647-93D1-A99C27C7EFDC}">
+    <text>I never thought it would be so low</text>
+  </threadedComment>
+  <threadedComment ref="G12" dT="2026-06-18T17:12:57.35" personId="{ED88F4F5-A552-4A41-970D-6B23DC2319F4}" id="{3A26E9AE-8B38-864D-BAF4-BA5D9C6E1DA4}">
+    <text>Maximum number of ducks</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Python is great</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Machine learning libraries</t>
-        </is>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D7" s="1">
+        <v>2019</v>
+      </c>
+      <c r="E7" s="1">
+        <v>120</v>
+      </c>
+      <c r="F7" s="1">
+        <v>80</v>
+      </c>
+      <c r="G7" s="1">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D8" s="1">
+        <v>2020</v>
+      </c>
+      <c r="E8" s="1">
+        <v>135</v>
+      </c>
+      <c r="F8" s="1">
+        <v>95</v>
+      </c>
+      <c r="G8" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D9" s="1">
+        <v>2021</v>
+      </c>
+      <c r="E9" s="1">
+        <v>150</v>
+      </c>
+      <c r="F9" s="1">
+        <v>100</v>
+      </c>
+      <c r="G9" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D10" s="1">
+        <v>2022</v>
+      </c>
+      <c r="E10" s="1">
+        <v>170</v>
+      </c>
+      <c r="F10" s="1">
+        <v>110</v>
+      </c>
+      <c r="G10" s="1">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D11" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E11" s="1">
+        <v>160</v>
+      </c>
+      <c r="F11" s="1">
+        <v>120</v>
+      </c>
+      <c r="G11" s="1">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D12" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E12" s="1">
+        <v>180</v>
+      </c>
+      <c r="F12" s="1">
+        <v>130</v>
+      </c>
+      <c r="G12" s="1">
+        <v>310</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>